<commit_message>
fix: restaura emails originais vagos, colunas exibem E-MAIL VAGO / ONEDRIVE
</commit_message>
<xml_diff>
--- a/Controle_/Acessos GTCON.xlsx
+++ b/Controle_/Acessos GTCON.xlsx
@@ -5267,7 +5267,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>E-MAIL VAGO</t>
+          <t>elaine@gtconbrasil.com.br</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -5279,7 +5279,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>E-MAIL VAGO</t>
+          <t>df30@gtconbrasil.com.br</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -5291,7 +5291,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>E-MAIL VAGO</t>
+          <t>df31@gtconbrasil.com.br</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -5303,7 +5303,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>E-MAIL VAGO</t>
+          <t>df8@gtconbrasil.com.br</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -5339,7 +5339,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>E-MAIL VAGO</t>
+          <t>df4@gtconbrasil.com.br</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -5375,7 +5375,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>E-MAIL VAGO</t>
+          <t>atendimento4@gtconbrasil.com.br</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -5411,7 +5411,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>E-MAIL VAGO</t>
+          <t>dc10@gtconbrasil.com.br</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -5423,7 +5423,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>E-MAIL VAGO</t>
+          <t>contabil.rj@gtconbrasil.com.br</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -5459,7 +5459,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>E-MAIL VAGO</t>
+          <t>dp15@gtconbrasil.com.br</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -5471,7 +5471,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>E-MAIL VAGO</t>
+          <t>dp5@gtconbrasil.com.br</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -5487,7 +5487,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>IMPLANTACAO DP</t>
+          <t>IMPLANTAÇÃO DP</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
@@ -5507,7 +5507,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>E-MAIL VAGO</t>
+          <t>implantacao3@gtconbrasil.com.br</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">

</xml_diff>

<commit_message>
feat: aba DP com colunas COLABORADOR, ANYDESK, E-MAIL, SENHA PADRAO ANYDESK, ONEDRIVE, CERTIFICADO GTCON, MAQUINA
</commit_message>
<xml_diff>
--- a/Controle_/Acessos GTCON.xlsx
+++ b/Controle_/Acessos GTCON.xlsx
@@ -5312,17 +5312,12 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" t="inlineStr"/>
-    </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
           <t>COMPLIANCE</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -5348,17 +5343,12 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr"/>
-      <c r="B11" t="inlineStr"/>
-    </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
           <t>ATENDIMENTO</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -5384,17 +5374,12 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr"/>
-      <c r="B15" t="inlineStr"/>
-    </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
           <t>CONTABIL</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -5432,17 +5417,12 @@
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr"/>
-      <c r="B20" t="inlineStr"/>
-    </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
           <t>DP</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -5480,17 +5460,12 @@
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="inlineStr"/>
-      <c r="B25" t="inlineStr"/>
-    </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
           <t>IMPLANTAÇÃO DP</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -6187,612 +6162,579 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor theme="4"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="19" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="12" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="39" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="24.42578125" bestFit="1" customWidth="1" min="4" max="4"/>
-    <col width="19.5703125" bestFit="1" customWidth="1" min="5" max="5"/>
-    <col width="20.42578125" bestFit="1" customWidth="1" min="6" max="6"/>
-    <col width="13.7109375" bestFit="1" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="25" t="inlineStr">
-        <is>
-          <t>DP</t>
-        </is>
-      </c>
-      <c r="B1" s="32" t="n"/>
-      <c r="C1" s="32" t="n"/>
-      <c r="D1" s="32" t="n"/>
-      <c r="E1" s="32" t="n"/>
-      <c r="F1" s="32" t="n"/>
-      <c r="G1" s="32" t="n"/>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>COLABORADOR</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>ANYDESK</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>E-MAIL</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>SENHA PADRAO ANYDESK</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>ONEDRIVE</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>CERTIFICADO GTCON</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>MAQUINA</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="27" t="inlineStr">
-        <is>
-          <t>COLABORADOR</t>
-        </is>
-      </c>
-      <c r="B2" s="27" t="inlineStr">
-        <is>
-          <t>ANYDESK</t>
-        </is>
-      </c>
-      <c r="C2" s="27" t="inlineStr">
-        <is>
-          <t>E-MAIL</t>
-        </is>
-      </c>
-      <c r="D2" s="27" t="inlineStr">
-        <is>
-          <t>SENHA PADRÃO ANYDESK</t>
-        </is>
-      </c>
-      <c r="E2" s="27" t="inlineStr">
-        <is>
-          <t>ONEDRIVE</t>
-        </is>
-      </c>
-      <c r="F2" s="20" t="inlineStr">
-        <is>
-          <t>CERTIFICADO GTCON</t>
-        </is>
-      </c>
-      <c r="G2" s="21" t="inlineStr">
-        <is>
-          <t>MAQUINA</t>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Emanuela </t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1607251811</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>dp3@gtconbrasil.com.br</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Gtcon#2024*</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>T#eC@1882</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Efg149375&amp;</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Emanuela </t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>1607251811</v>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>dp3@gtconbrasil.com.br</t>
-        </is>
-      </c>
-      <c r="D3" s="1" t="inlineStr">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Gabriella</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>512261603</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>dp.1@gtconbrasil.com.br</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
         <is>
           <t>Gtcon#2024*</t>
         </is>
       </c>
-      <c r="E3" s="1" t="inlineStr">
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>R!816723436344on</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Josimara Alves</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>1007205611</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>dp10@gtconbrasil.com.br</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Gtcon#2024*</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Z#876179077002af</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>1234</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Karina Alves</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>1514474252</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>dp12@gtconbrasil.com.br</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Gtcon#2024*</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>X(420695250462at</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>25130710Fa@</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Lidiane Oliveira</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>597358922</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>dp16@gtconbrasil.com.br</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Gtcon#2025</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>GTCON25</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Livia</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>626237333</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>dp2@gtconbrasil.com.br</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Gtcon#2024*</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
         <is>
           <t>T#eC@1882</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>Efg149375&amp;</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Gabriella</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>512261603</v>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>dp.1@gtconbrasil.com.br</t>
-        </is>
-      </c>
-      <c r="D4" s="1" t="inlineStr">
+      <c r="G7" t="n">
+        <v>1234</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Luísa </t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>1876934276</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>dp14@gtconbrasil.com.br</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
         <is>
           <t>Gtcon#2024*</t>
         </is>
       </c>
-      <c r="E4" s="1" t="inlineStr">
-        <is>
-          <t>R!816723436344on</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Q)904672906240ux</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Josimara Alves</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>1007205611</v>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>dp10@gtconbrasil.com.br</t>
-        </is>
-      </c>
-      <c r="D5" s="1" t="inlineStr">
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>GTCON25</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Luiz Gustavo </t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>493882728</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>dp21@gtconbrasil.com.br</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
         <is>
           <t>Gtcon#2024*</t>
         </is>
       </c>
-      <c r="E5" s="1" t="inlineStr">
-        <is>
-          <t>Z#876179077002af</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>G%367822712641ar</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="G5" s="4" t="n">
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>GTCON25</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Monique</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>1478923107</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>dp17@gtconbrasil.com.br</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Gtcon#2024*</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>H$975428139147ot</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>GTCON25</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Raphaela</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>1555081951</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>dp7@gtconbrasil.com.br</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Gtcon#2025*</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>T#eC@1881</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>1967</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Thais</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>997159970</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>dp11@gtconbrasil.com.br</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Gtcon#2024*</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Z$707010893181az</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
         <v>1234</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Karina Alves</t>
-        </is>
-      </c>
-      <c r="B6" s="1" t="n">
-        <v>1514474252</v>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>dp12@gtconbrasil.com.br</t>
-        </is>
-      </c>
-      <c r="D6" s="1" t="inlineStr">
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Vivian</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>1803850864</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>departamentopessoal@gtconbrasil.com.br</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
         <is>
           <t>Gtcon#2024*</t>
         </is>
       </c>
-      <c r="E6" s="1" t="inlineStr">
-        <is>
-          <t>X(420695250462at</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Q.092954551838uz</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>25130710Fa@</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Lidiane Oliveira</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>597358922</v>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>dp16@gtconbrasil.com.br</t>
-        </is>
-      </c>
-      <c r="D7" s="1" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E7" s="1" t="inlineStr">
-        <is>
-          <t>Gtcon#2025</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lorran </t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>1607251811</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>dp13@gtconbrasil.com.br</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Gtcon#2024*</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>N$049996617795ub</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>GTCON25</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Livia</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>626237333</v>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>dp2@gtconbrasil.com.br</t>
-        </is>
-      </c>
-      <c r="D8" s="1" t="inlineStr">
-        <is>
-          <t>Gtcon#2024*</t>
-        </is>
-      </c>
-      <c r="E8" s="1" t="inlineStr">
-        <is>
-          <t>T#eC@1882</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="G8" s="4" t="n">
-        <v>1234</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Luísa </t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="n">
-        <v>1876934276</v>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>dp14@gtconbrasil.com.br</t>
-        </is>
-      </c>
-      <c r="D9" s="1" t="inlineStr">
-        <is>
-          <t>Gtcon#2024*</t>
-        </is>
-      </c>
-      <c r="E9" s="1" t="inlineStr">
-        <is>
-          <t>Q)904672906240ux</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>GTCON25</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Luiz Gustavo </t>
-        </is>
-      </c>
-      <c r="B10" s="1" t="n">
-        <v>493882728</v>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>dp21@gtconbrasil.com.br</t>
-        </is>
-      </c>
-      <c r="D10" s="1" t="inlineStr">
-        <is>
-          <t>Gtcon#2024*</t>
-        </is>
-      </c>
-      <c r="E10" s="1" t="inlineStr">
-        <is>
-          <t>G%367822712641ar</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>GTCON25</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Monique</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>1478923107</v>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>dp17@gtconbrasil.com.br</t>
-        </is>
-      </c>
-      <c r="D11" s="1" t="inlineStr">
-        <is>
-          <t>Gtcon#2024*</t>
-        </is>
-      </c>
-      <c r="E11" s="1" t="inlineStr">
-        <is>
-          <t>H$975428139147ot</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>GTCON25</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Raphaela</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>1555081951</v>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>dp7@gtconbrasil.com.br</t>
-        </is>
-      </c>
-      <c r="D12" s="1" t="inlineStr">
-        <is>
-          <t>Gtcon#2025*</t>
-        </is>
-      </c>
-      <c r="E12" s="1" t="inlineStr">
-        <is>
-          <t>T#eC@1881</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="G12" s="4" t="n">
-        <v>1967</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Thais</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>997159970</v>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>dp11@gtconbrasil.com.br</t>
-        </is>
-      </c>
-      <c r="D13" s="1" t="inlineStr">
-        <is>
-          <t>Gtcon#2024*</t>
-        </is>
-      </c>
-      <c r="E13" s="1" t="inlineStr">
-        <is>
-          <t>Z$707010893181az</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="G13" s="4" t="n">
-        <v>1234</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Vivian</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>1803850864</v>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>departamentopessoal@gtconbrasil.com.br</t>
-        </is>
-      </c>
-      <c r="D14" s="1" t="inlineStr">
-        <is>
-          <t>Gtcon#2024*</t>
-        </is>
-      </c>
-      <c r="E14" s="1" t="inlineStr">
-        <is>
-          <t>Q.092954551838uz</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lorran </t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>1607251811</v>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>dp13@gtconbrasil.com.br</t>
-        </is>
-      </c>
-      <c r="D15" s="1" t="inlineStr">
-        <is>
-          <t>Gtcon#2024*</t>
-        </is>
-      </c>
-      <c r="E15" s="1" t="inlineStr">
-        <is>
-          <t>N$049996617795ub</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>GTCON25</t>
-        </is>
-      </c>
+      <c r="A15" t="inlineStr"/>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>ROMULO</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="25" t="inlineStr">
-        <is>
-          <t>ROMULO</t>
-        </is>
-      </c>
-      <c r="B17" s="32" t="n"/>
-      <c r="C17" s="32" t="n"/>
-      <c r="D17" s="32" t="n"/>
-      <c r="E17" s="32" t="n"/>
-      <c r="F17" s="32" t="n"/>
-      <c r="G17" s="8" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="27" t="inlineStr">
-        <is>
-          <t>COLABORADOR</t>
-        </is>
-      </c>
-      <c r="B18" s="27" t="inlineStr">
-        <is>
-          <t>ANYDESK</t>
-        </is>
-      </c>
-      <c r="C18" s="27" t="inlineStr">
-        <is>
-          <t>E-MAIL</t>
-        </is>
-      </c>
-      <c r="D18" s="27" t="inlineStr">
-        <is>
-          <t>SENHA ANYDESK</t>
-        </is>
-      </c>
-      <c r="E18" s="27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SENHA UNICO </t>
-        </is>
-      </c>
-      <c r="F18" s="27" t="inlineStr">
-        <is>
-          <t>ONEDRIVE</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="n">
-        <v>569215440</v>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>569215440</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
         <is>
           <t>administrativo1@gtconbrasil.com.br</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>Rdestac25</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>GTCON</t>
         </is>
       </c>
-      <c r="F19" s="1" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>F*415203413144ot</t>
         </is>
       </c>
+      <c r="G17" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A17:F17"/>
-    <mergeCell ref="A1:G1"/>
-  </mergeCells>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" display="mailto:dp10@grupoteccon.com.br" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" display="mailto:dp12@grupoteccon.com.br" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" display="mailto:dp7@grupoteccon.com.br" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" display="mailto:dp11@grupoteccon.com.br" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId10"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
feat: aba Comercial padronizada com mesmas colunas
</commit_message>
<xml_diff>
--- a/Controle_/Acessos GTCON.xlsx
+++ b/Controle_/Acessos GTCON.xlsx
@@ -3442,70 +3442,90 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor theme="0" tint="-0.3499862666707358"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="15.7109375" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="12" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="38.7109375" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="24.42578125" bestFit="1" customWidth="1" min="4" max="4"/>
-    <col width="19.42578125" bestFit="1" customWidth="1" min="5" max="5"/>
-    <col width="20.42578125" bestFit="1" customWidth="1" min="6" max="6"/>
-    <col width="9.7109375" bestFit="1" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="30" t="inlineStr">
-        <is>
-          <t>COMERCIAL</t>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>COLABORADOR</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>ANYDESK</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>E-MAIL</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>SENHA PADRAO ANYDESK</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>ONEDRIVE</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>CERTIFICADO GTCON</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>MAQUINA</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="27" t="inlineStr">
-        <is>
-          <t>COLABORADOR</t>
-        </is>
-      </c>
-      <c r="B2" s="27" t="inlineStr">
-        <is>
-          <t>ANYDESK</t>
-        </is>
-      </c>
-      <c r="C2" s="27" t="inlineStr">
-        <is>
-          <t>E-MAIL</t>
-        </is>
-      </c>
-      <c r="D2" s="27" t="inlineStr">
-        <is>
-          <t>SENHA PADRÃO ANYDESK</t>
-        </is>
-      </c>
-      <c r="E2" s="27" t="inlineStr">
-        <is>
-          <t>ONEDRIVE</t>
-        </is>
-      </c>
-      <c r="F2" s="20" t="inlineStr">
-        <is>
-          <t>CERTIFICADO GTCON</t>
-        </is>
-      </c>
-      <c r="G2" s="21" t="inlineStr">
-        <is>
-          <t>MAQUINA</t>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ayrton</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>ayrtonjunior@gtconbrasil.com.br</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>V#254258672703ol</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>NÃO UTILIZA</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Ayrton</t>
+          <t xml:space="preserve">Daniel </t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -3515,7 +3535,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ayrtonjunior@gtconbrasil.com.br</t>
+          <t>comercial1@gtconbrasil.com.br</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -3523,9 +3543,9 @@
           <t>-</t>
         </is>
       </c>
-      <c r="E3" s="1" t="inlineStr">
-        <is>
-          <t>V#254258672703ol</t>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>K*227143754197op</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -3533,7 +3553,7 @@
           <t>NÃO UTILIZA</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -3542,7 +3562,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Daniel </t>
+          <t>Ellen</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -3552,7 +3572,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>comercial1@gtconbrasil.com.br</t>
+          <t>ellen@gtconbrasil.com.br</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -3562,7 +3582,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>K*227143754197op</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -3570,7 +3590,7 @@
           <t>NÃO UTILIZA</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -3579,7 +3599,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Ellen</t>
+          <t>Felipe Rodrigues</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -3589,7 +3609,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ellen@gtconbrasil.com.br</t>
+          <t>comercial@gtconbrasil.com.br</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -3599,7 +3619,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t xml:space="preserve">K%886307565079ur </t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -3607,7 +3627,7 @@
           <t>NÃO UTILIZA</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -3616,7 +3636,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Felipe Rodrigues</t>
+          <t>Fernando</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -3626,7 +3646,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>comercial@gtconbrasil.com.br</t>
+          <t>fernandosantos@gtconbrasil.com.br</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -3634,9 +3654,9 @@
           <t>-</t>
         </is>
       </c>
-      <c r="E6" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">K%886307565079ur </t>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -3644,7 +3664,7 @@
           <t>NÃO UTILIZA</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -3653,27 +3673,27 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Fernando</t>
+          <t>Kaique</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1543419339</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>fernandosantos@gtconbrasil.com.br</t>
+          <t>comercial2@gtconbrasil.com.br</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Gtcon#2024*</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>T@881445245502ag</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -3681,7 +3701,7 @@
           <t>NÃO UTILIZA</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -3690,25 +3710,27 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Kaique</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>1543419339</v>
+          <t>Marco</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>comercial2@gtconbrasil.com.br</t>
-        </is>
-      </c>
-      <c r="D8" s="1" t="inlineStr">
-        <is>
-          <t>Gtcon#2024*</t>
+          <t>marco@gtconbrasil.com.br</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>T@881445245502ag</t>
+          <t>L&amp;085495255261os</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -3716,7 +3738,7 @@
           <t>NÃO UTILIZA</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -3725,7 +3747,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Marco</t>
+          <t>Mauricio</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -3735,7 +3757,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>marco@gtconbrasil.com.br</t>
+          <t>mauriciooliveira@gtconbrasil.com.br</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -3743,9 +3765,9 @@
           <t>-</t>
         </is>
       </c>
-      <c r="E9" s="1" t="inlineStr">
-        <is>
-          <t>L&amp;085495255261os</t>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>F$398479054850oz</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -3753,7 +3775,7 @@
           <t>NÃO UTILIZA</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -3762,7 +3784,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Mauricio</t>
+          <t>Ranieri</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -3772,17 +3794,13 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>mauriciooliveira@gtconbrasil.com.br</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E10" s="1" t="inlineStr">
-        <is>
-          <t>F$398479054850oz</t>
+          <t>ranieri@gtconbrasil.com.br</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>M%121117676032uf</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -3790,16 +3808,12 @@
           <t>NÃO UTILIZA</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Ranieri</t>
+          <t>Walter</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -3809,12 +3823,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ranieri@gtconbrasil.com.br</t>
+          <t>walter.leite@gtconbrasil.com.br</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>M%121117676032uf</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -3822,56 +3841,14 @@
           <t>NÃO UTILIZA</t>
         </is>
       </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Walter</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>walter.leite@gtconbrasil.com.br</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>NÃO UTILIZA</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
-  </mergeCells>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId5"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -4075,7 +4052,6 @@
           <t>Dominio</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>adm.dominio@gtconbrasil.com.br</t>
@@ -4256,7 +4232,6 @@
           <t>Onvio/G-click | Integração</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
           <t>integracaogclick@gtconbrasil.com.br</t>

</xml_diff>